<commit_message>
Redeploy con ajustes para el mvp
</commit_message>
<xml_diff>
--- a/data/productos.xlsx
+++ b/data/productos.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{111FB73A-ED7F-4748-AC1B-B939C25BA5C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{431A0AB7-30CB-417F-A293-F40ACAD73D6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="70">
   <si>
     <t>Id</t>
   </si>
@@ -67,7 +67,7 @@
     <t>Activo</t>
   </si>
   <si>
-    <t>BP-2030-D</t>
+    <t>BP-1x10x2</t>
   </si>
   <si>
     <t>Bolsa transparente</t>
@@ -82,34 +82,43 @@
     <t>Paquete x 100 unidades</t>
   </si>
   <si>
+    <t>bolsa-product.webp</t>
+  </si>
+  <si>
+    <t>Sí</t>
+  </si>
+  <si>
+    <t>BP-1-1/8x10x2</t>
+  </si>
+  <si>
+    <t>1 1/8</t>
+  </si>
+  <si>
+    <t>Intermedio</t>
+  </si>
+  <si>
     <t>bolsa-transparente.webp</t>
   </si>
   <si>
-    <t>Sí</t>
-  </si>
-  <si>
-    <t>BP-2030-I</t>
-  </si>
-  <si>
-    <t>Intermedio</t>
-  </si>
-  <si>
-    <t>BP-2030-G</t>
+    <t>No</t>
+  </si>
+  <si>
+    <t>BP-1-1/4x10x2</t>
+  </si>
+  <si>
+    <t>1</t>
   </si>
   <si>
     <t>Grueso</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>BP-3040-D</t>
-  </si>
-  <si>
-    <t>BP-3040-I</t>
-  </si>
-  <si>
-    <t>BN-4050-G</t>
+    <t>BP-1-1/2x10x2-E</t>
+  </si>
+  <si>
+    <t>BP-1-1/2x10x2-N</t>
+  </si>
+  <si>
+    <t>BP-1-3/4x10x2-E</t>
   </si>
   <si>
     <t>Bolsa negra</t>
@@ -121,7 +130,7 @@
     <t>bolsa-negra.webp</t>
   </si>
   <si>
-    <t>BC-2535-I</t>
+    <t>BP-1-3/4x10x2-N</t>
   </si>
   <si>
     <t>Bolsa de color</t>
@@ -133,10 +142,79 @@
     <t>bolsa-blanca.webp</t>
   </si>
   <si>
-    <t>BP-5060-G</t>
+    <t>BP-2x10x2-E</t>
   </si>
   <si>
     <t>Bolsa transparente grande</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>BP-2x10x2-N</t>
+  </si>
+  <si>
+    <t>BP-2-1/8x10x2</t>
+  </si>
+  <si>
+    <t>BP-2-1/4x10x2</t>
+  </si>
+  <si>
+    <t>BP-2-1/2x10x2</t>
+  </si>
+  <si>
+    <t>BP-2-3/4x10x2</t>
+  </si>
+  <si>
+    <t>BP-3x10x2</t>
+  </si>
+  <si>
+    <t>BP-3-1/4x10x2</t>
+  </si>
+  <si>
+    <t>BP-3-1/2x10x2</t>
+  </si>
+  <si>
+    <t>BP-3-3/4x10x2</t>
+  </si>
+  <si>
+    <t>BP-4x10x2</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>BP-4-1/4x10x2</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>BP-4-1/2x10x2</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>BP-5x10x2</t>
+  </si>
+  <si>
+    <t>BP-5-1/2x10x2</t>
+  </si>
+  <si>
+    <t>BP-6x10x2</t>
+  </si>
+  <si>
+    <t>BP-6-1/2x10x2</t>
+  </si>
+  <si>
+    <t>BP-7x10x2</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>BP-8x10x2</t>
   </si>
   <si>
     <t>Sí/No</t>
@@ -219,7 +297,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -228,6 +306,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -248,7 +329,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProductosTable" displayName="ProductosTable" ref="A1:K9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProductosTable" displayName="ProductosTable" ref="A1:K27">
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Id"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Codigo"/>
@@ -415,7 +496,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -474,11 +555,11 @@
       <c r="C2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2">
-        <v>20</v>
+      <c r="D2" s="4">
+        <v>1</v>
       </c>
       <c r="E2" s="2">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>13</v>
@@ -509,15 +590,15 @@
       <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="2">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="2">
-        <v>30</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="G3" s="2" t="s">
         <v>14</v>
       </c>
@@ -525,10 +606,10 @@
         <v>15</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>17</v>
@@ -539,19 +620,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="2">
-        <v>20</v>
+      <c r="D4" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="E4" s="2">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>14</v>
@@ -574,16 +655,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2">
-        <v>30</v>
+      <c r="D5" s="4" t="s">
+        <v>24</v>
       </c>
       <c r="E5" s="2">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>13</v>
@@ -595,7 +676,7 @@
         <v>15</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>22</v>
@@ -609,19 +690,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2">
-        <v>30</v>
-      </c>
       <c r="E6" s="2">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>14</v>
@@ -630,10 +711,10 @@
         <v>15</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>17</v>
@@ -644,28 +725,28 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="2">
-        <v>40</v>
-      </c>
-      <c r="E7" s="2">
-        <v>50</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="G7" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>22</v>
@@ -679,31 +760,31 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="2">
-        <v>25</v>
+        <v>33</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1</v>
       </c>
       <c r="E8" s="2">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>32</v>
-      </c>
       <c r="J8" s="2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>17</v>
@@ -714,33 +795,663 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9" s="2">
+        <v>37</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="2">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="16.5">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="4">
+        <v>2</v>
+      </c>
+      <c r="E10" s="2">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="16.5">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2</v>
+      </c>
+      <c r="E11" s="2">
+        <v>10</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="16.5">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="4">
+        <v>2</v>
+      </c>
+      <c r="E12" s="2">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="16.5">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2</v>
+      </c>
+      <c r="E13" s="2">
+        <v>10</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="16.5">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="4">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2">
+        <v>10</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="16.5">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="4">
+        <v>3</v>
+      </c>
+      <c r="E15" s="2">
+        <v>10</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="16.5">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="4">
+        <v>3</v>
+      </c>
+      <c r="E16" s="2">
+        <v>10</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="16.5">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="4">
+        <v>3</v>
+      </c>
+      <c r="E17" s="2">
+        <v>10</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="16.5">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="4">
+        <v>3</v>
+      </c>
+      <c r="E18" s="2">
+        <v>10</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="16.5">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E19" s="2">
+        <v>10</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="16.5">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E9" s="2">
+      <c r="C20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="E20" s="2">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="16.5">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E21" s="2">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="16.5">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="4">
+        <v>5</v>
+      </c>
+      <c r="E22" s="2">
+        <v>10</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="16.5">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="4">
+        <v>5</v>
+      </c>
+      <c r="E23" s="2">
+        <v>10</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="16.5">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="4">
+        <v>6</v>
+      </c>
+      <c r="E24" s="2">
+        <v>10</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="16.5">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="2">
+        <v>10</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K25" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="16.5">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="2">
+        <v>10</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="16.5">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="K9" s="2" t="s">
+      <c r="C27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="4">
+        <v>8</v>
+      </c>
+      <c r="E27" s="2">
+        <v>10</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K27" s="2" t="s">
         <v>17</v>
       </c>
     </row>
@@ -756,19 +1467,19 @@
           <x14:formula1>
             <xm:f>Catalogos!$A$2:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>F2:F501</xm:sqref>
+          <xm:sqref>F2:F519</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000001000000}">
           <x14:formula1>
             <xm:f>Catalogos!$B$2:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>G2:G501</xm:sqref>
+          <xm:sqref>G2:G519</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000002000000}">
           <x14:formula1>
             <xm:f>Catalogos!$C$2:$C$3</xm:f>
           </x14:formula1>
-          <xm:sqref>J2:K501</xm:sqref>
+          <xm:sqref>J2:K519</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -795,10 +1506,10 @@
         <v>6</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>61</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>36</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -812,53 +1523,53 @@
         <v>17</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>37</v>
+        <v>63</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>41</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>43</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>